<commit_message>
Add dates next to day names in bag count export
- Dates appear in row 2 next to each day (e.g., Monday 03/30)
- Format: MM/DD
- Automatically calculates based on current week
</commit_message>
<xml_diff>
--- a/data/Cycle_Bag_Count_2026_W14.xlsx
+++ b/data/Cycle_Bag_Count_2026_W14.xlsx
@@ -985,28 +985,48 @@
       <c r="B2" s="35" t="s">
         <v>62</v>
       </c>
-      <c r="C2" s="34"/>
+      <c r="C2" s="34" t="inlineStr">
+        <is>
+          <t>03/30</t>
+        </is>
+      </c>
       <c r="D2" s="34"/>
       <c r="F2" s="35" t="s">
         <v>61</v>
       </c>
-      <c r="G2" s="35"/>
+      <c r="G2" s="35" t="inlineStr">
+        <is>
+          <t>03/31</t>
+        </is>
+      </c>
       <c r="H2" s="35"/>
       <c r="J2" s="35" t="s">
         <v>60</v>
       </c>
-      <c r="K2" s="34"/>
+      <c r="K2" s="34" t="inlineStr">
+        <is>
+          <t>04/01</t>
+        </is>
+      </c>
       <c r="L2" s="34"/>
       <c r="M2" s="36"/>
       <c r="N2" s="35" t="s">
         <v>59</v>
       </c>
-      <c r="O2" s="34"/>
+      <c r="O2" s="34" t="inlineStr">
+        <is>
+          <t>04/02</t>
+        </is>
+      </c>
       <c r="P2" s="34"/>
       <c r="R2" s="35" t="s">
         <v>58</v>
       </c>
-      <c r="S2" s="34"/>
+      <c r="S2" s="34" t="inlineStr">
+        <is>
+          <t>04/03</t>
+        </is>
+      </c>
       <c r="T2" s="34"/>
     </row>
     <row r="3" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
@@ -1832,28 +1852,48 @@
       <c r="B2" s="35" t="s">
         <v>62</v>
       </c>
-      <c r="C2" s="34"/>
+      <c r="C2" s="34" t="inlineStr">
+        <is>
+          <t>03/30</t>
+        </is>
+      </c>
       <c r="D2" s="34"/>
       <c r="F2" s="35" t="s">
         <v>61</v>
       </c>
-      <c r="G2" s="35"/>
+      <c r="G2" s="35" t="inlineStr">
+        <is>
+          <t>03/31</t>
+        </is>
+      </c>
       <c r="H2" s="35"/>
       <c r="J2" s="35" t="s">
         <v>60</v>
       </c>
-      <c r="K2" s="34"/>
+      <c r="K2" s="34" t="inlineStr">
+        <is>
+          <t>04/01</t>
+        </is>
+      </c>
       <c r="L2" s="34"/>
       <c r="M2" s="36"/>
       <c r="N2" s="35" t="s">
         <v>59</v>
       </c>
-      <c r="O2" s="34"/>
+      <c r="O2" s="34" t="inlineStr">
+        <is>
+          <t>04/02</t>
+        </is>
+      </c>
       <c r="P2" s="34"/>
       <c r="R2" s="35" t="s">
         <v>58</v>
       </c>
-      <c r="S2" s="34"/>
+      <c r="S2" s="34" t="inlineStr">
+        <is>
+          <t>04/03</t>
+        </is>
+      </c>
       <c r="T2" s="34"/>
     </row>
     <row r="3" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">

</xml_diff>

<commit_message>
Fix: update both sheets in single pass to prevent data loss
- Previous code was overwriting sheet1 when updating sheet2
- Now reads all files once, updates both sheets, writes once
</commit_message>
<xml_diff>
--- a/data/Cycle_Bag_Count_2026_W14.xlsx
+++ b/data/Cycle_Bag_Count_2026_W14.xlsx
@@ -964,12 +964,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{34A602E7-DCF8-4DBB-9A82-740C7064C3FD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac xr xr2 xr3" ns2:uid="{34A602E7-DCF8-4DBB-9A82-740C7064C3FD}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B2:T40"/>
-  <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.85546875" customWidth="1"/>
     <col min="5" max="5" width="2.42578125" customWidth="1"/>
@@ -981,7 +981,7 @@
     <col min="18" max="18" width="11.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="2" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="35" t="s">
         <v>62</v>
       </c>
@@ -1029,7 +1029,7 @@
       </c>
       <c r="T2" s="34"/>
     </row>
-    <row r="3" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="3" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>57</v>
       </c>
@@ -1076,7 +1076,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="4" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="18" t="s">
         <v>54</v>
       </c>
@@ -1115,7 +1115,7 @@
       <c r="S4" s="27"/>
       <c r="T4" s="26"/>
     </row>
-    <row r="5" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="5" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="15"/>
       <c r="C5" s="31"/>
       <c r="D5" s="13"/>
@@ -1130,7 +1130,7 @@
       <c r="O5" s="31"/>
       <c r="P5" s="13"/>
     </row>
-    <row r="6" spans="2:20" ns3:dyDescent="0.25">
+    <row r="6" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B6" s="15"/>
       <c r="C6" s="14" t="s">
         <v>46</v>
@@ -1169,7 +1169,7 @@
       </c>
       <c r="T6" s="16"/>
     </row>
-    <row r="7" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="7" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="15"/>
       <c r="C7" s="14" t="s">
         <v>42</v>
@@ -1195,7 +1195,7 @@
       <c r="S7" s="31"/>
       <c r="T7" s="13"/>
     </row>
-    <row r="8" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="8" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="12"/>
       <c r="C8" s="11"/>
       <c r="D8" s="29">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="T8" s="13"/>
     </row>
-    <row r="9" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="9" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F9" s="30" t="s">
         <v>41</v>
       </c>
@@ -1238,7 +1238,7 @@
       <c r="S9" s="31"/>
       <c r="T9" s="13"/>
     </row>
-    <row r="10" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="10" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B10" s="18" t="s">
         <v>40</v>
       </c>
@@ -1274,14 +1274,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="11" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="15"/>
       <c r="C11" s="14" t="s">
         <v>37</v>
       </c>
       <c r="D11" s="13"/>
     </row>
-    <row r="12" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="12" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="12"/>
       <c r="C12" s="11"/>
       <c r="D12" s="10">
@@ -1321,7 +1321,7 @@
       </c>
       <c r="T12" s="16"/>
     </row>
-    <row r="13" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="13" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="J13" s="15"/>
       <c r="K13" s="14">
         <v>2</v>
@@ -1338,7 +1338,7 @@
       <c r="S13" s="31"/>
       <c r="T13" s="13"/>
     </row>
-    <row r="14" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="14" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="18" t="s">
         <v>32</v>
       </c>
@@ -1376,7 +1376,7 @@
       </c>
       <c r="T14" s="13"/>
     </row>
-    <row r="15" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="15" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="15"/>
       <c r="C15" s="14" t="s">
         <v>28</v>
@@ -1401,7 +1401,7 @@
       <c r="S15" s="31"/>
       <c r="T15" s="13"/>
     </row>
-    <row r="16" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="16" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="15"/>
       <c r="C16" s="14" t="s">
         <v>27</v>
@@ -1431,7 +1431,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="17" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="12"/>
       <c r="C17" s="11"/>
       <c r="D17" s="10">
@@ -1453,7 +1453,7 @@
       </c>
       <c r="P17" s="13"/>
     </row>
-    <row r="18" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="18" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F18" s="9" t="s">
         <v>65</v>
       </c>
@@ -1478,7 +1478,7 @@
       </c>
       <c r="T18" s="16"/>
     </row>
-    <row r="19" spans="2:20" ns3:dyDescent="0.25">
+    <row r="19" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B19" s="18" t="s">
         <v>23</v>
       </c>
@@ -1504,7 +1504,7 @@
       </c>
       <c r="T19" s="13"/>
     </row>
-    <row r="20" spans="2:20" ns3:dyDescent="0.25">
+    <row r="20" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B20" s="15"/>
       <c r="C20" s="14" t="s">
         <v>21</v>
@@ -1526,7 +1526,7 @@
       </c>
       <c r="T20" s="13"/>
     </row>
-    <row r="21" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="21" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="12"/>
       <c r="C21" s="11"/>
       <c r="D21" s="10">
@@ -1552,12 +1552,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="22" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="P22">
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="23" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B23" s="21" t="s">
         <v>20</v>
       </c>
@@ -1588,7 +1588,7 @@
       </c>
       <c r="T23" s="16"/>
     </row>
-    <row r="24" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="24" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B24" s="20"/>
       <c r="C24" s="14" t="s">
         <v>16</v>
@@ -1600,7 +1600,7 @@
       </c>
       <c r="T24" s="13"/>
     </row>
-    <row r="25" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="25" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B25" s="20"/>
       <c r="C25" s="14" t="s">
         <v>15</v>
@@ -1622,7 +1622,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="2:20" ns3:dyDescent="0.25">
+    <row r="26" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B26" s="20"/>
       <c r="C26" s="14" t="s">
         <v>12</v>
@@ -1636,7 +1636,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="27" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="27" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B27" s="19"/>
       <c r="C27" s="11"/>
       <c r="D27" s="29">
@@ -1659,7 +1659,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="28" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="J28" s="25"/>
       <c r="K28" s="24" t="s">
         <v>10</v>
@@ -1668,7 +1668,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="29" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B29" s="28" t="s">
         <v>9</v>
       </c>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="L29" s="23"/>
     </row>
-    <row r="30" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="30" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="J30" s="22"/>
       <c r="K30" s="11"/>
       <c r="L30" s="10">
@@ -1690,7 +1690,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="2:20" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="31" spans="2:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="21" t="s">
         <v>7</v>
       </c>
@@ -1701,7 +1701,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="32" spans="2:20" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="32" spans="2:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="20"/>
       <c r="C32" s="14" t="s">
         <v>5</v>
@@ -1716,7 +1716,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="33" spans="2:15" ht="15" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="33" spans="2:15" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B33" s="19"/>
       <c r="C33" s="11"/>
       <c r="D33" s="10">
@@ -1724,8 +1724,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="2:15" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3"/>
-    <row r="35" spans="2:15" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="34" spans="2:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="35" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="18" t="s">
         <v>4</v>
       </c>
@@ -1736,14 +1736,14 @@
         <v>10</v>
       </c>
     </row>
-    <row r="36" spans="2:15" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="36" spans="2:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="15"/>
       <c r="C36" s="14" t="s">
         <v>2</v>
       </c>
       <c r="D36" s="13"/>
     </row>
-    <row r="37" spans="2:15" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="37" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B37" s="12"/>
       <c r="C37" s="11"/>
       <c r="D37" s="10">
@@ -1751,8 +1751,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="2:15" ht="15.75" thickBot="1" ns3:dyDescent="0.3"/>
-    <row r="39" spans="2:15" ht="21.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="38" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="39" spans="2:15" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="9" t="s">
         <v>65</v>
       </c>
@@ -1773,7 +1773,7 @@
       <c r="N39" s="6"/>
       <c r="O39" s="5"/>
     </row>
-    <row r="40" spans="2:15" ht="21" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="40" spans="2:15" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="J40" s="4"/>
       <c r="K40" s="3"/>
       <c r="L40" s="2"/>
@@ -1831,12 +1831,12 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{EC5CAEEA-E072-4740-85F2-234693AA0991}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac xr xr2 xr3" ns2:uid="{EC5CAEEA-E072-4740-85F2-234693AA0991}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B2:T40"/>
-  <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.85546875" customWidth="1"/>
     <col min="5" max="5" width="2.42578125" customWidth="1"/>
@@ -1848,7 +1848,7 @@
     <col min="18" max="18" width="11.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="2" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="35" t="s">
         <v>62</v>
       </c>
@@ -1896,7 +1896,7 @@
       </c>
       <c r="T2" s="34"/>
     </row>
-    <row r="3" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="3" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>57</v>
       </c>
@@ -1943,7 +1943,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="4" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="4" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="18" t="s">
         <v>54</v>
       </c>
@@ -1980,7 +1980,7 @@
       <c r="S4" s="27"/>
       <c r="T4" s="26"/>
     </row>
-    <row r="5" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="5" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="15"/>
       <c r="C5" s="31"/>
       <c r="D5" s="13"/>
@@ -1995,7 +1995,7 @@
       <c r="O5" s="31"/>
       <c r="P5" s="13"/>
     </row>
-    <row r="6" spans="2:20" ns3:dyDescent="0.25">
+    <row r="6" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B6" s="15"/>
       <c r="C6" s="14" t="s">
         <v>46</v>
@@ -2032,7 +2032,7 @@
       </c>
       <c r="T6" s="16"/>
     </row>
-    <row r="7" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="7" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="15"/>
       <c r="C7" s="14" t="s">
         <v>42</v>
@@ -2060,7 +2060,7 @@
       <c r="S7" s="31"/>
       <c r="T7" s="13"/>
     </row>
-    <row r="8" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="8" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="12"/>
       <c r="C8" s="11"/>
       <c r="D8" s="29">
@@ -2086,7 +2086,7 @@
       </c>
       <c r="T8" s="13"/>
     </row>
-    <row r="9" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="9" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F9" s="30" t="s">
         <v>41</v>
       </c>
@@ -2105,7 +2105,7 @@
       <c r="S9" s="31"/>
       <c r="T9" s="13"/>
     </row>
-    <row r="10" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="10" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B10" s="18" t="s">
         <v>40</v>
       </c>
@@ -2139,7 +2139,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="11" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="15"/>
       <c r="C11" s="14" t="s">
         <v>37</v>
@@ -2148,7 +2148,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="12" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="12" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="12"/>
       <c r="C12" s="11"/>
       <c r="D12" s="10">
@@ -2186,7 +2186,7 @@
       </c>
       <c r="T12" s="16"/>
     </row>
-    <row r="13" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="13" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="J13" s="15"/>
       <c r="K13" s="14">
         <v>2</v>
@@ -2203,7 +2203,7 @@
       <c r="S13" s="31"/>
       <c r="T13" s="13"/>
     </row>
-    <row r="14" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="14" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="18" t="s">
         <v>32</v>
       </c>
@@ -2241,7 +2241,7 @@
       </c>
       <c r="T14" s="13"/>
     </row>
-    <row r="15" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="15" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="15"/>
       <c r="C15" s="14" t="s">
         <v>28</v>
@@ -2266,7 +2266,7 @@
       <c r="S15" s="31"/>
       <c r="T15" s="13"/>
     </row>
-    <row r="16" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="16" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="15"/>
       <c r="C16" s="14" t="s">
         <v>27</v>
@@ -2294,7 +2294,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="17" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="12"/>
       <c r="C17" s="11"/>
       <c r="D17" s="10">
@@ -2316,7 +2316,7 @@
       </c>
       <c r="P17" s="13"/>
     </row>
-    <row r="18" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="18" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F18" s="9" t="s">
         <v>1</v>
       </c>
@@ -2341,7 +2341,7 @@
       </c>
       <c r="T18" s="16"/>
     </row>
-    <row r="19" spans="2:20" ns3:dyDescent="0.25">
+    <row r="19" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B19" s="18" t="s">
         <v>23</v>
       </c>
@@ -2369,7 +2369,7 @@
       </c>
       <c r="T19" s="13"/>
     </row>
-    <row r="20" spans="2:20" ns3:dyDescent="0.25">
+    <row r="20" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B20" s="15"/>
       <c r="C20" s="14" t="s">
         <v>21</v>
@@ -2391,7 +2391,7 @@
       </c>
       <c r="T20" s="13"/>
     </row>
-    <row r="21" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="21" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="12"/>
       <c r="C21" s="11"/>
       <c r="D21" s="10">
@@ -2417,8 +2417,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3"/>
-    <row r="23" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="22" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="23" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B23" s="21" t="s">
         <v>20</v>
       </c>
@@ -2449,7 +2449,7 @@
       </c>
       <c r="T23" s="16"/>
     </row>
-    <row r="24" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="24" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B24" s="20"/>
       <c r="C24" s="14" t="s">
         <v>16</v>
@@ -2463,7 +2463,7 @@
       </c>
       <c r="T24" s="13"/>
     </row>
-    <row r="25" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="25" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B25" s="20"/>
       <c r="C25" s="14" t="s">
         <v>15</v>
@@ -2487,7 +2487,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="2:20" ns3:dyDescent="0.25">
+    <row r="26" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B26" s="20"/>
       <c r="C26" s="14" t="s">
         <v>12</v>
@@ -2503,7 +2503,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="27" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="27" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B27" s="19"/>
       <c r="C27" s="11"/>
       <c r="D27" s="29">
@@ -2526,7 +2526,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="28" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="J28" s="25"/>
       <c r="K28" s="24" t="s">
         <v>10</v>
@@ -2535,7 +2535,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="29" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="29" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B29" s="28" t="s">
         <v>9</v>
       </c>
@@ -2549,7 +2549,7 @@
       </c>
       <c r="L29" s="23"/>
     </row>
-    <row r="30" spans="2:20" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="30" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="J30" s="22"/>
       <c r="K30" s="11"/>
       <c r="L30" s="10">
@@ -2557,7 +2557,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="2:20" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="31" spans="2:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="21" t="s">
         <v>7</v>
       </c>
@@ -2568,7 +2568,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="32" spans="2:20" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="32" spans="2:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="20"/>
       <c r="C32" s="14" t="s">
         <v>5</v>
@@ -2585,7 +2585,7 @@
         <v>11512</v>
       </c>
     </row>
-    <row r="33" spans="2:15" ht="15" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="33" spans="2:15" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B33" s="19"/>
       <c r="C33" s="11"/>
       <c r="D33" s="10">
@@ -2593,8 +2593,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="2:15" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3"/>
-    <row r="35" spans="2:15" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="34" spans="2:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="35" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="18" t="s">
         <v>4</v>
       </c>
@@ -2605,14 +2605,14 @@
         <v>297</v>
       </c>
     </row>
-    <row r="36" spans="2:15" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="36" spans="2:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="15"/>
       <c r="C36" s="14" t="s">
         <v>2</v>
       </c>
       <c r="D36" s="13"/>
     </row>
-    <row r="37" spans="2:15" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="37" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B37" s="12"/>
       <c r="C37" s="11"/>
       <c r="D37" s="10">
@@ -2620,8 +2620,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="2:15" ht="15.75" thickBot="1" ns3:dyDescent="0.3"/>
-    <row r="39" spans="2:15" ht="21.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="38" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="39" spans="2:15" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="9" t="s">
         <v>1</v>
       </c>
@@ -2642,7 +2642,7 @@
       <c r="N39" s="6"/>
       <c r="O39" s="5"/>
     </row>
-    <row r="40" spans="2:15" ht="21" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="40" spans="2:15" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="J40" s="4"/>
       <c r="K40" s="3"/>
       <c r="L40" s="2"/>

</xml_diff>